<commit_message>
Log T2 session 2026-06-11 (Pull/Core + wrist-modified OAHS)
</commit_message>
<xml_diff>
--- a/Training_2_Sheets.xlsx
+++ b/Training_2_Sheets.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="758">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1416" uniqueCount="766">
   <si>
     <t>B6 — Performance-Block Dashboard (Google-Sheets-Version)</t>
   </si>
@@ -1684,6 +1684,30 @@
   </si>
   <si>
     <t>Satz1: 40 kg x3; Satz2-4: 35 kg x4; RPE 8-9</t>
+  </si>
+  <si>
+    <t>Rowing-Maschine, horizontal, solide</t>
+  </si>
+  <si>
+    <t>Latzug-Maschine</t>
+  </si>
+  <si>
+    <t>Reverse Butterfly</t>
+  </si>
+  <si>
+    <t>Face Pull; Gewicht ~30 kg, noch pruefen</t>
+  </si>
+  <si>
+    <t>30s</t>
+  </si>
+  <si>
+    <t>Core-Finisher, 3x30s Hollow</t>
+  </si>
+  <si>
+    <t>Parallettes links, ging gut; wegen Handgelenk modifiziert</t>
+  </si>
+  <si>
+    <t>Boden rechts mit Abstuetzen/Halten; Handgelenk - separat bewerten</t>
   </si>
   <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -6684,7 +6708,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -7418,6 +7442,289 @@
       </c>
       <c r="P18" s="6">
         <f>IF($B18="","",$B18&amp;"_W"&amp;$C18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
+      <c r="A19" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="E19" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D19,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G19" s="6">
+        <v>3</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="I19" s="6">
+        <v>90</v>
+      </c>
+      <c r="J19" s="6">
+        <v>8</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="P19" s="6">
+        <f>IF($B19="","",$B19&amp;"_W"&amp;$C19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16">
+      <c r="A20" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="E20" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D20,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G20" s="6">
+        <v>3</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="I20" s="6">
+        <v>70</v>
+      </c>
+      <c r="J20" s="6">
+        <v>8</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="P20" s="6">
+        <f>IF($B20="","",$B20&amp;"_W"&amp;$C20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16">
+      <c r="A21" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>424</v>
+      </c>
+      <c r="E21" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D21,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G21" s="6">
+        <v>3</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="I21" s="6">
+        <v>35</v>
+      </c>
+      <c r="J21" s="6">
+        <v>7</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="P21" s="6">
+        <f>IF($B21="","",$B21&amp;"_W"&amp;$C21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
+      <c r="A22" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" s="6">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="E22" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D22,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G22" s="6">
+        <v>2</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="I22" s="6">
+        <v>30</v>
+      </c>
+      <c r="J22" s="6">
+        <v>7</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="P22" s="6">
+        <f>IF($B22="","",$B22&amp;"_W"&amp;$C22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
+      <c r="A23" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="6">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="E23" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D23,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G23" s="6">
+        <v>3</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="M23" s="6">
+        <v>30</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="P23" s="6">
+        <f>IF($B23="","",$B23&amp;"_W"&amp;$C23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
+      <c r="A24" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="E24" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D24,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="G24" s="6">
+        <v>2</v>
+      </c>
+      <c r="I24" s="6">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6">
+        <v>6</v>
+      </c>
+      <c r="K24" s="6">
+        <v>2</v>
+      </c>
+      <c r="L24" s="6">
+        <v>4</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="P24" s="6">
+        <f>IF($B24="","",$B24&amp;"_W"&amp;$C24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16">
+      <c r="A25" s="20">
+        <v>46184</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="E25" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D25,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G25" s="6">
+        <v>2</v>
+      </c>
+      <c r="I25" s="6">
+        <v>0</v>
+      </c>
+      <c r="J25" s="6">
+        <v>6</v>
+      </c>
+      <c r="K25" s="6">
+        <v>2</v>
+      </c>
+      <c r="L25" s="6">
+        <v>3</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="P25" s="6">
+        <f>IF($B25="","",$B25&amp;"_W"&amp;$C25)</f>
         <v>0</v>
       </c>
     </row>
@@ -7483,7 +7790,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7494,20 +7801,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>562</v>
+        <v>570</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -7516,21 +7823,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>556</v>
+        <v>564</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>557</v>
+        <v>565</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -7539,7 +7846,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>558</v>
+        <v>566</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -7547,7 +7854,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>559</v>
+        <v>567</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -7555,7 +7862,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>560</v>
+        <v>568</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -7564,7 +7871,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -7573,7 +7880,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -7587,27 +7894,27 @@
         <v>83</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>565</v>
+        <v>573</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>566</v>
+        <v>574</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>569</v>
+        <v>577</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>570</v>
+        <v>578</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>571</v>
+        <v>579</v>
       </c>
       <c r="B14" s="21">
         <v>250</v>
@@ -7629,7 +7936,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>572</v>
+        <v>580</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -7656,12 +7963,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>574</v>
+        <v>582</v>
       </c>
       <c r="B16" s="21">
         <v>200</v>
@@ -7683,12 +7990,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>575</v>
+        <v>583</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>576</v>
+        <v>584</v>
       </c>
       <c r="B17" s="21">
         <v>150</v>
@@ -7710,12 +8017,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>577</v>
+        <v>585</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="B18" s="21">
         <v>100</v>
@@ -7737,7 +8044,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>579</v>
+        <v>587</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -7764,12 +8071,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>580</v>
+        <v>588</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -7780,7 +8087,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>582</v>
+        <v>590</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -7791,7 +8098,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>583</v>
+        <v>591</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -7802,7 +8109,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>584</v>
+        <v>592</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -7813,7 +8120,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -7858,7 +8165,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>586</v>
+        <v>594</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7867,7 +8174,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -7876,109 +8183,109 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>588</v>
+        <v>596</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>589</v>
+        <v>597</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>591</v>
+        <v>599</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>592</v>
+        <v>600</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>597</v>
+        <v>605</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>598</v>
+        <v>606</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>603</v>
+        <v>611</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>605</v>
+        <v>613</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>607</v>
+        <v>615</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>608</v>
+        <v>616</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>613</v>
+        <v>621</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -7987,7 +8294,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -7996,7 +8303,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -8005,7 +8312,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -8014,7 +8321,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -8023,7 +8330,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -8032,7 +8339,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="4" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -8041,7 +8348,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -8050,19 +8357,19 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="7" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -8070,16 +8377,16 @@
         <v>65</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>631</v>
+        <v>639</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -8087,16 +8394,16 @@
         <v>47</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>636</v>
+        <v>644</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -8104,16 +8411,16 @@
         <v>33</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>640</v>
+        <v>648</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>641</v>
+        <v>649</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -8121,21 +8428,21 @@
         <v>32</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>643</v>
+        <v>651</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>646</v>
+        <v>654</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="26" t="s">
-        <v>647</v>
+        <v>655</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -8144,7 +8451,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -8153,7 +8460,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -8162,7 +8469,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -8171,7 +8478,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -8180,7 +8487,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -8189,7 +8496,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -8198,7 +8505,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="5" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -8207,104 +8514,104 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="7" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -8362,7 +8669,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8372,7 +8679,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -8397,12 +8704,12 @@
         <v>151</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Skill90",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Push",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8427,7 +8734,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Pull",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8452,7 +8759,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Legs",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8477,7 +8784,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS('B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8502,7 +8809,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS('B6_Training_Log'!$N$2:$N$1000,'B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8527,7 +8834,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8552,7 +8859,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8677,7 +8984,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Core",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8702,7 +9009,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$J$2:$J$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -8727,7 +9034,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$K$2:$K$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -8777,7 +9084,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS('B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8821,7 +9128,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8829,7 +9136,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8837,13 +9144,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -8852,10 +9159,10 @@
         <v>519</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -8864,10 +9171,10 @@
         <v>520</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -8876,10 +9183,10 @@
         <v>521</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -8888,10 +9195,10 @@
         <v>358</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -8900,10 +9207,10 @@
         <v>361</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -8912,10 +9219,10 @@
         <v>522</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -8924,10 +9231,10 @@
         <v>523</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -8936,10 +9243,10 @@
         <v>524</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -8948,10 +9255,10 @@
         <v>525</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -8960,10 +9267,10 @@
         <v>526</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -8972,10 +9279,10 @@
         <v>527</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -8984,10 +9291,10 @@
         <v>528</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -8996,10 +9303,10 @@
         <v>529</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -9008,10 +9315,10 @@
         <v>530</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -9020,10 +9327,10 @@
         <v>90</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -9032,16 +9339,16 @@
         <v>531</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -9049,7 +9356,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9057,7 +9364,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9065,7 +9372,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9073,7 +9380,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -9081,7 +9388,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -9089,7 +9396,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9097,7 +9404,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -9105,13 +9412,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -9120,10 +9427,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>736</v>
+        <v>744</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>737</v>
+        <v>745</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -9132,10 +9439,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>738</v>
+        <v>746</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -9144,10 +9451,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -9156,40 +9463,40 @@
         <v>297</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="13" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>746</v>
+        <v>754</v>
       </c>
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="13" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>748</v>
+        <v>756</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>750</v>
+        <v>758</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -9197,7 +9504,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -9205,7 +9512,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>752</v>
+        <v>760</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -9213,7 +9520,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>753</v>
+        <v>761</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -9221,7 +9528,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>754</v>
+        <v>762</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -9229,7 +9536,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>755</v>
+        <v>763</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -9237,7 +9544,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>756</v>
+        <v>764</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -9245,7 +9552,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>757</v>
+        <v>765</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>

<commit_message>
Log T3 session 2026-06-12 (legs DOMS-limited + parallettes holds)
</commit_message>
<xml_diff>
--- a/Training_2_Sheets.xlsx
+++ b/Training_2_Sheets.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1416" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="770">
   <si>
     <t>B6 — Performance-Block Dashboard (Google-Sheets-Version)</t>
   </si>
@@ -1710,6 +1710,21 @@
     <t>Boden rechts mit Abstuetzen/Halten; Handgelenk - separat bewerten</t>
   </si>
   <si>
+    <t>Parallettes-Holds zu Beginn; Handgelenk-Ziehen mild/kein Problem; andere Hand Druck-/Greifproblem (evtl. Unterarm/Hand ueberreizt)</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>runter von 45 auf 40 kg wegen starkem Muskelkater (Vorwoche); Quads links brannten; Qualitaet nicht ideal</t>
+  </si>
+  <si>
+    <t>12-15</t>
+  </si>
+  <si>
+    <t>12/12/15</t>
+  </si>
+  <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
   </si>
   <si>
@@ -2293,9 +2308,6 @@
   </si>
   <si>
     <t>ExerciseID=pseudo_planche_pushup, Category(auto)=Planche, Sets=3, Reps_or_Scheme=8, TopRPE=8</t>
-  </si>
-  <si>
-    <t>6</t>
   </si>
   <si>
     <t>T3 Woche 1, Hinge mit Dowel 3 Reps Ruecken 1, dann Beinpresse 3 mal 12 mit 120 Kilo RPE 7.</t>
@@ -6708,7 +6720,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -7725,6 +7737,200 @@
       </c>
       <c r="P25" s="6">
         <f>IF($B25="","",$B25&amp;"_W"&amp;$C25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="A26" s="20">
+        <v>46185</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="6">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="E26" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D26,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G26" s="6">
+        <v>3</v>
+      </c>
+      <c r="I26" s="6">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6">
+        <v>1</v>
+      </c>
+      <c r="L26" s="6">
+        <v>3</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="P26" s="6">
+        <f>IF($B26="","",$B26&amp;"_W"&amp;$C26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16">
+      <c r="A27" s="20">
+        <v>46185</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="6">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="E27" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D27,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G27" s="6">
+        <v>3</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="I27" s="6">
+        <v>40</v>
+      </c>
+      <c r="J27" s="6">
+        <v>8</v>
+      </c>
+      <c r="O27" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="P27" s="6">
+        <f>IF($B27="","",$B27&amp;"_W"&amp;$C27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16">
+      <c r="A28" s="20">
+        <v>46185</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="E28" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D28,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G28" s="6">
+        <v>3</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="I28" s="6">
+        <v>60</v>
+      </c>
+      <c r="J28" s="6">
+        <v>7</v>
+      </c>
+      <c r="P28" s="6">
+        <f>IF($B28="","",$B28&amp;"_W"&amp;$C28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16">
+      <c r="A29" s="20">
+        <v>46185</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" s="6">
+        <v>1</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="E29" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D29,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G29" s="6">
+        <v>3</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="I29" s="6">
+        <v>50</v>
+      </c>
+      <c r="J29" s="6">
+        <v>7</v>
+      </c>
+      <c r="P29" s="6">
+        <f>IF($B29="","",$B29&amp;"_W"&amp;$C29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16">
+      <c r="A30" s="20">
+        <v>46185</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="E30" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$43,MATCH($D30,'B6_Exercise_Library'!$A$4:$A$43,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="G30" s="6">
+        <v>3</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="I30" s="6">
+        <v>70</v>
+      </c>
+      <c r="J30" s="6">
+        <v>7</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="P30" s="6">
+        <f>IF($B30="","",$B30&amp;"_W"&amp;$C30)</f>
         <v>0</v>
       </c>
     </row>
@@ -7790,7 +7996,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7801,20 +8007,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -7823,21 +8029,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -7846,7 +8052,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -7854,7 +8060,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -7862,7 +8068,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -7871,7 +8077,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -7880,7 +8086,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -7894,27 +8100,27 @@
         <v>83</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="B14" s="21">
         <v>250</v>
@@ -7936,7 +8142,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -7963,12 +8169,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="B16" s="21">
         <v>200</v>
@@ -7990,12 +8196,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="B17" s="21">
         <v>150</v>
@@ -8017,12 +8223,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="B18" s="21">
         <v>100</v>
@@ -8044,7 +8250,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8071,12 +8277,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -8087,7 +8293,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -8098,7 +8304,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -8109,7 +8315,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -8120,7 +8326,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -8165,7 +8371,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8174,7 +8380,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8183,109 +8389,109 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -8294,7 +8500,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -8303,7 +8509,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -8312,7 +8518,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -8321,7 +8527,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -8330,7 +8536,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -8339,7 +8545,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="4" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -8348,7 +8554,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -8357,19 +8563,19 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="7" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -8377,16 +8583,16 @@
         <v>65</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -8394,16 +8600,16 @@
         <v>47</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -8411,16 +8617,16 @@
         <v>33</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -8428,21 +8634,21 @@
         <v>32</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="26" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -8451,7 +8657,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -8460,7 +8666,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -8469,7 +8675,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -8478,7 +8684,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -8487,7 +8693,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -8496,7 +8702,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -8505,7 +8711,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="5" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -8514,104 +8720,104 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="7" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="B37" s="27" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="B41" s="27" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -8669,7 +8875,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8679,7 +8885,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -8704,12 +8910,12 @@
         <v>151</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Skill90",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Push",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8734,7 +8940,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Pull",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8759,7 +8965,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Legs",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8784,7 +8990,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS('B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8809,7 +9015,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS('B6_Training_Log'!$N$2:$N$1000,'B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8834,7 +9040,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8859,7 +9065,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -8984,7 +9190,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Core",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9009,7 +9215,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$J$2:$J$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -9034,7 +9240,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$K$2:$K$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -9084,7 +9290,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS('B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9128,7 +9334,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9136,7 +9342,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -9144,13 +9350,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -9159,10 +9365,10 @@
         <v>519</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -9171,10 +9377,10 @@
         <v>520</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -9183,10 +9389,10 @@
         <v>521</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>709</v>
+        <v>714</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -9195,10 +9401,10 @@
         <v>358</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -9207,10 +9413,10 @@
         <v>361</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -9219,10 +9425,10 @@
         <v>522</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -9231,10 +9437,10 @@
         <v>523</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -9243,10 +9449,10 @@
         <v>524</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -9255,10 +9461,10 @@
         <v>525</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -9267,10 +9473,10 @@
         <v>526</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -9279,10 +9485,10 @@
         <v>527</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -9291,10 +9497,10 @@
         <v>528</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -9303,10 +9509,10 @@
         <v>529</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -9315,10 +9521,10 @@
         <v>530</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -9327,10 +9533,10 @@
         <v>90</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -9339,16 +9545,16 @@
         <v>531</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -9356,7 +9562,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9364,7 +9570,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9372,7 +9578,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9380,7 +9586,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -9388,7 +9594,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -9396,7 +9602,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9404,7 +9610,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -9412,13 +9618,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -9427,10 +9633,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -9439,10 +9645,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>747</v>
+        <v>752</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -9451,10 +9657,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -9463,40 +9669,40 @@
         <v>297</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="13" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="D36" s="4"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="13" t="s">
-        <v>755</v>
+        <v>561</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -9504,7 +9710,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -9512,7 +9718,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -9520,7 +9726,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -9528,7 +9734,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -9536,7 +9742,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -9544,7 +9750,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -9552,7 +9758,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>

<commit_message>
Log T2 session 2026-06-19 (W2: home skill microdose + pull/core)
</commit_message>
<xml_diff>
--- a/Training_2_Sheets.xlsx
+++ b/Training_2_Sheets.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1451" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="780">
   <si>
     <t>B6 — Performance-Block Dashboard (Google-Sheets-Version)</t>
   </si>
@@ -1738,6 +1738,21 @@
   </si>
   <si>
     <t>Ruhetag: Handgelenk/Unterarm + Bein-DOMS schonen; leichte Mobility/Soft-Tissue, gut essen</t>
+  </si>
+  <si>
+    <t>Handstand-Mikrodosis zu Hause; mehrere solide Holds, 6+ s links</t>
+  </si>
+  <si>
+    <t>auch ein paar solide Holds rechts</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Seated Row Maschine, 45 kg/Seite</t>
+  </si>
+  <si>
+    <t>Core-Finisher, 3x30s</t>
   </si>
   <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -6779,7 +6794,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -8018,6 +8033,274 @@
       </c>
       <c r="P31" s="6">
         <f>IF($B31="","",$B31&amp;"_W"&amp;$C31)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="A32" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="6">
+        <v>2</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="E32" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D32,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="G32" s="6">
+        <v>3</v>
+      </c>
+      <c r="I32" s="6">
+        <v>0</v>
+      </c>
+      <c r="L32" s="6">
+        <v>4</v>
+      </c>
+      <c r="M32" s="6">
+        <v>6</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="P32" s="6">
+        <f>IF($B32="","",$B32&amp;"_W"&amp;$C32)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16">
+      <c r="A33" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" s="6">
+        <v>2</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="E33" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D33,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="G33" s="6">
+        <v>2</v>
+      </c>
+      <c r="I33" s="6">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6">
+        <v>3</v>
+      </c>
+      <c r="O33" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="P33" s="6">
+        <f>IF($B33="","",$B33&amp;"_W"&amp;$C33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16">
+      <c r="A34" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" s="6">
+        <v>2</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="E34" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D34,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G34" s="6">
+        <v>4</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="I34" s="6">
+        <v>70</v>
+      </c>
+      <c r="J34" s="6">
+        <v>7</v>
+      </c>
+      <c r="P34" s="6">
+        <f>IF($B34="","",$B34&amp;"_W"&amp;$C34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16">
+      <c r="A35" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="6">
+        <v>2</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E35" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D35,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G35" s="6">
+        <v>4</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I35" s="6">
+        <v>90</v>
+      </c>
+      <c r="J35" s="6">
+        <v>7</v>
+      </c>
+      <c r="O35" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="P35" s="6">
+        <f>IF($B35="","",$B35&amp;"_W"&amp;$C35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16">
+      <c r="A36" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="6">
+        <v>2</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="E36" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D36,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G36" s="6">
+        <v>3</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="I36" s="6">
+        <v>35</v>
+      </c>
+      <c r="J36" s="6">
+        <v>7</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="P36" s="6">
+        <f>IF($B36="","",$B36&amp;"_W"&amp;$C36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16">
+      <c r="A37" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" s="6">
+        <v>2</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="E37" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D37,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G37" s="6">
+        <v>3</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="I37" s="6">
+        <v>25</v>
+      </c>
+      <c r="J37" s="6">
+        <v>7</v>
+      </c>
+      <c r="P37" s="6">
+        <f>IF($B37="","",$B37&amp;"_W"&amp;$C37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16">
+      <c r="A38" s="21">
+        <v>46192</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="6">
+        <v>2</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="E38" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D38,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G38" s="6">
+        <v>3</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="M38" s="6">
+        <v>30</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="P38" s="6">
+        <f>IF($B38="","",$B38&amp;"_W"&amp;$C38)</f>
         <v>0</v>
       </c>
     </row>
@@ -8083,7 +8366,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8094,20 +8377,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -8116,21 +8399,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -8139,7 +8422,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -8147,7 +8430,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -8155,7 +8438,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -8164,7 +8447,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -8173,7 +8456,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -8187,27 +8470,27 @@
         <v>84</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="B14" s="22">
         <v>250</v>
@@ -8229,7 +8512,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -8256,12 +8539,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="B16" s="22">
         <v>200</v>
@@ -8283,12 +8566,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="B17" s="22">
         <v>150</v>
@@ -8310,12 +8593,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="B18" s="22">
         <v>100</v>
@@ -8337,7 +8620,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8364,12 +8647,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -8380,7 +8663,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -8391,7 +8674,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -8402,7 +8685,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -8413,7 +8696,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -8458,7 +8741,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8467,7 +8750,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8476,109 +8759,109 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -8587,7 +8870,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -8596,7 +8879,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -8605,7 +8888,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -8614,7 +8897,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -8623,7 +8906,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -8632,7 +8915,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="4" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -8641,7 +8924,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -8650,19 +8933,19 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="7" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -8670,16 +8953,16 @@
         <v>65</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -8687,16 +8970,16 @@
         <v>47</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -8704,16 +8987,16 @@
         <v>33</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -8721,21 +9004,21 @@
         <v>32</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="27" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
@@ -8744,7 +9027,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -8753,7 +9036,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -8762,7 +9045,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -8771,7 +9054,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -8780,7 +9063,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -8789,7 +9072,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -8798,7 +9081,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="5" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -8807,104 +9090,104 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="7" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="B36" s="28" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -8962,7 +9245,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8972,7 +9255,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -8997,12 +9280,12 @@
         <v>152</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Skill90",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Push",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9027,7 +9310,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Pull",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9052,7 +9335,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Legs",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9077,7 +9360,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS('B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9102,7 +9385,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS('B6_Training_Log'!$N$2:$N$1000,'B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9127,7 +9410,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9152,7 +9435,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9277,7 +9560,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Core",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9302,7 +9585,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$J$2:$J$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -9327,7 +9610,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$K$2:$K$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -9377,7 +9660,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>709</v>
+        <v>714</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS('B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9421,7 +9704,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9429,7 +9712,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -9437,13 +9720,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -9452,10 +9735,10 @@
         <v>523</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -9464,10 +9747,10 @@
         <v>524</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -9476,10 +9759,10 @@
         <v>525</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -9488,10 +9771,10 @@
         <v>359</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -9500,10 +9783,10 @@
         <v>362</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -9512,10 +9795,10 @@
         <v>526</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -9524,10 +9807,10 @@
         <v>527</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -9536,10 +9819,10 @@
         <v>528</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -9548,10 +9831,10 @@
         <v>529</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -9560,10 +9843,10 @@
         <v>530</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -9572,10 +9855,10 @@
         <v>531</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -9584,10 +9867,10 @@
         <v>532</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -9596,10 +9879,10 @@
         <v>533</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -9608,10 +9891,10 @@
         <v>534</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -9620,10 +9903,10 @@
         <v>91</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -9632,16 +9915,16 @@
         <v>535</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -9649,7 +9932,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9657,7 +9940,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9665,7 +9948,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9673,7 +9956,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>747</v>
+        <v>752</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -9681,7 +9964,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -9689,7 +9972,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9697,7 +9980,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -9705,13 +9988,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -9720,10 +10003,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -9732,10 +10015,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -9744,10 +10027,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -9756,22 +10039,22 @@
         <v>298</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="14" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="D36" s="4"/>
     </row>
@@ -9780,16 +10063,16 @@
         <v>565</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -9797,7 +10080,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -9805,7 +10088,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -9813,7 +10096,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -9821,7 +10104,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -9829,7 +10112,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -9837,7 +10120,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>773</v>
+        <v>778</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -9845,7 +10128,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>

<commit_message>
Log T4/T5 (W2) + T1 (W3) sessions
</commit_message>
<xml_diff>
--- a/Training_2_Sheets.xlsx
+++ b/Training_2_Sheets.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="799">
   <si>
     <t>B6 — Performance-Block Dashboard (Google-Sheets-Version)</t>
   </si>
@@ -1753,6 +1753,63 @@
   </si>
   <si>
     <t>Core-Finisher, 3x30s</t>
+  </si>
+  <si>
+    <t>Unsupported Flag-Lean + 1 Arm geloest, zurueck zum Center; links gut</t>
+  </si>
+  <si>
+    <t>Unsupported Flag-Lean; rechts semi, aber gute Kontrolle</t>
+  </si>
+  <si>
+    <t>Straddle Flag Hold, 1-3s freeze; links gut, rechts wechselhaft</t>
+  </si>
+  <si>
+    <t>S1:3voll, S2:2voll, S3-4:2-3 Neg</t>
+  </si>
+  <si>
+    <t>Super Tag: volle Reps locker @RPE7 obwohl nur Negative geplant; 3 saubere Reps am Stueck in Satz1</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Feet elevated Pike Push-up</t>
+  </si>
+  <si>
+    <t>Chest-supported Row Maschine</t>
+  </si>
+  <si>
+    <t>2-3 Negativ</t>
+  </si>
+  <si>
+    <t>Negativ-Mikro wie geplant</t>
+  </si>
+  <si>
+    <t>12/10/10</t>
+  </si>
+  <si>
+    <t>Kabelzug; 2x80kg, 2x75kg</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>nur bedacht/ruhig moeglich; 3-5s Holds mit Exit zurueck; Pisiform gereizt</t>
+  </si>
+  <si>
+    <t>wechselhaft, nur gehalten wenn moeglich; Pisiform gereizt</t>
+  </si>
+  <si>
+    <t>2 schwere Einzel-Reps + 1 fail</t>
+  </si>
+  <si>
+    <t>Peak-Tag aber Regeneration 1/5 + Hitze, alles uebersaeuert; Doubles geplant; nach 2 schweren Singles + Fail (Koerperspannung weg) 90 abgebrochen</t>
+  </si>
+  <si>
+    <t>statt Tuck Planche (zu wenig Kraft heute); 4x6</t>
+  </si>
+  <si>
+    <t>ermuedet, Gewicht reduziert auf 35 kg</t>
   </si>
   <si>
     <t>B6 — Nutrition Targets (Maintenance, KEIN Defizit)</t>
@@ -6794,7 +6851,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -8301,6 +8358,763 @@
       </c>
       <c r="P38" s="6">
         <f>IF($B38="","",$B38&amp;"_W"&amp;$C38)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="A39" s="21">
+        <v>46194</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C39" s="6">
+        <v>2</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="E39" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D39,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="G39" s="6">
+        <v>5</v>
+      </c>
+      <c r="I39" s="6">
+        <v>0</v>
+      </c>
+      <c r="L39" s="6">
+        <v>4</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="P39" s="6">
+        <f>IF($B39="","",$B39&amp;"_W"&amp;$C39)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="A40" s="21">
+        <v>46194</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C40" s="6">
+        <v>2</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="E40" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D40,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="G40" s="6">
+        <v>5</v>
+      </c>
+      <c r="I40" s="6">
+        <v>0</v>
+      </c>
+      <c r="L40" s="6">
+        <v>3</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="P40" s="6">
+        <f>IF($B40="","",$B40&amp;"_W"&amp;$C40)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16">
+      <c r="A41" s="21">
+        <v>46194</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C41" s="6">
+        <v>2</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="E41" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D41,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G41" s="6">
+        <v>4</v>
+      </c>
+      <c r="I41" s="6">
+        <v>0</v>
+      </c>
+      <c r="L41" s="6">
+        <v>3</v>
+      </c>
+      <c r="M41" s="6">
+        <v>3</v>
+      </c>
+      <c r="O41" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="P41" s="6">
+        <f>IF($B41="","",$B41&amp;"_W"&amp;$C41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16">
+      <c r="A42" s="21">
+        <v>46194</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C42" s="6">
+        <v>2</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="E42" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D42,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G42" s="6">
+        <v>4</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="I42" s="6">
+        <v>0</v>
+      </c>
+      <c r="J42" s="6">
+        <v>7</v>
+      </c>
+      <c r="L42" s="6">
+        <v>4</v>
+      </c>
+      <c r="N42" s="6">
+        <v>5</v>
+      </c>
+      <c r="O42" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="P42" s="6">
+        <f>IF($B42="","",$B42&amp;"_W"&amp;$C42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16">
+      <c r="A43" s="21">
+        <v>46194</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" s="6">
+        <v>2</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="E43" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D43,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G43" s="6">
+        <v>3</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="I43" s="6">
+        <v>0</v>
+      </c>
+      <c r="J43" s="6">
+        <v>7</v>
+      </c>
+      <c r="O43" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="P43" s="6">
+        <f>IF($B43="","",$B43&amp;"_W"&amp;$C43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16">
+      <c r="A44" s="21">
+        <v>46194</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C44" s="6">
+        <v>2</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E44" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D44,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G44" s="6">
+        <v>3</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I44" s="6">
+        <v>90</v>
+      </c>
+      <c r="J44" s="6">
+        <v>7</v>
+      </c>
+      <c r="O44" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="P44" s="6">
+        <f>IF($B44="","",$B44&amp;"_W"&amp;$C44)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16">
+      <c r="A45" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C45" s="6">
+        <v>2</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="E45" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D45,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G45" s="6">
+        <v>3</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="I45" s="6">
+        <v>0</v>
+      </c>
+      <c r="J45" s="6">
+        <v>6</v>
+      </c>
+      <c r="L45" s="6">
+        <v>4</v>
+      </c>
+      <c r="O45" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="P45" s="6">
+        <f>IF($B45="","",$B45&amp;"_W"&amp;$C45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16">
+      <c r="A46" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C46" s="6">
+        <v>2</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="E46" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D46,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G46" s="6">
+        <v>3</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="I46" s="6">
+        <v>0</v>
+      </c>
+      <c r="J46" s="6">
+        <v>8</v>
+      </c>
+      <c r="P46" s="6">
+        <f>IF($B46="","",$B46&amp;"_W"&amp;$C46)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="A47" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" s="6">
+        <v>2</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="E47" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D47,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G47" s="6">
+        <v>4</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I47" s="6">
+        <v>70</v>
+      </c>
+      <c r="J47" s="6">
+        <v>7</v>
+      </c>
+      <c r="P47" s="6">
+        <f>IF($B47="","",$B47&amp;"_W"&amp;$C47)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16">
+      <c r="A48" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C48" s="6">
+        <v>2</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E48" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D48,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G48" s="6">
+        <v>4</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I48" s="6">
+        <v>80</v>
+      </c>
+      <c r="J48" s="6">
+        <v>7</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="P48" s="6">
+        <f>IF($B48="","",$B48&amp;"_W"&amp;$C48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16">
+      <c r="A49" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" s="6">
+        <v>2</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="E49" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D49,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G49" s="6">
+        <v>3</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="I49" s="6">
+        <v>8</v>
+      </c>
+      <c r="J49" s="6">
+        <v>7</v>
+      </c>
+      <c r="P49" s="6">
+        <f>IF($B49="","",$B49&amp;"_W"&amp;$C49)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16">
+      <c r="A50" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C50" s="6">
+        <v>2</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="E50" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D50,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G50" s="6">
+        <v>3</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="I50" s="6">
+        <v>30</v>
+      </c>
+      <c r="J50" s="6">
+        <v>7</v>
+      </c>
+      <c r="P50" s="6">
+        <f>IF($B50="","",$B50&amp;"_W"&amp;$C50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16">
+      <c r="A51" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C51" s="6">
+        <v>2</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="E51" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D51,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G51" s="6">
+        <v>3</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I51" s="6">
+        <v>23.5</v>
+      </c>
+      <c r="J51" s="6">
+        <v>7</v>
+      </c>
+      <c r="P51" s="6">
+        <f>IF($B51="","",$B51&amp;"_W"&amp;$C51)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16">
+      <c r="A52" s="21">
+        <v>46196</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C52" s="6">
+        <v>2</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="E52" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D52,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G52" s="6">
+        <v>3</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="I52" s="6">
+        <v>16.5</v>
+      </c>
+      <c r="J52" s="6">
+        <v>7</v>
+      </c>
+      <c r="P52" s="6">
+        <f>IF($B52="","",$B52&amp;"_W"&amp;$C52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16">
+      <c r="A53" s="21">
+        <v>46198</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C53" s="6">
+        <v>3</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="E53" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D53,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="G53" s="6">
+        <v>5</v>
+      </c>
+      <c r="I53" s="6">
+        <v>0</v>
+      </c>
+      <c r="K53" s="6">
+        <v>2</v>
+      </c>
+      <c r="L53" s="6">
+        <v>3</v>
+      </c>
+      <c r="M53" s="6">
+        <v>5</v>
+      </c>
+      <c r="O53" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="P53" s="6">
+        <f>IF($B53="","",$B53&amp;"_W"&amp;$C53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16">
+      <c r="A54" s="21">
+        <v>46198</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="6">
+        <v>3</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="E54" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D54,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="G54" s="6">
+        <v>5</v>
+      </c>
+      <c r="I54" s="6">
+        <v>0</v>
+      </c>
+      <c r="K54" s="6">
+        <v>2</v>
+      </c>
+      <c r="L54" s="6">
+        <v>2</v>
+      </c>
+      <c r="M54" s="6">
+        <v>2</v>
+      </c>
+      <c r="O54" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="P54" s="6">
+        <f>IF($B54="","",$B54&amp;"_W"&amp;$C54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16">
+      <c r="A55" s="21">
+        <v>46198</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C55" s="6">
+        <v>3</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="E55" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D55,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G55" s="6">
+        <v>3</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="I55" s="6">
+        <v>0</v>
+      </c>
+      <c r="J55" s="6">
+        <v>9</v>
+      </c>
+      <c r="L55" s="6">
+        <v>2</v>
+      </c>
+      <c r="N55" s="6">
+        <v>0</v>
+      </c>
+      <c r="O55" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="P55" s="6">
+        <f>IF($B55="","",$B55&amp;"_W"&amp;$C55)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16">
+      <c r="A56" s="21">
+        <v>46198</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C56" s="6">
+        <v>3</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="E56" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D56,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G56" s="6">
+        <v>4</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="I56" s="6">
+        <v>0</v>
+      </c>
+      <c r="J56" s="6">
+        <v>8</v>
+      </c>
+      <c r="O56" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="P56" s="6">
+        <f>IF($B56="","",$B56&amp;"_W"&amp;$C56)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16">
+      <c r="A57" s="21">
+        <v>46198</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C57" s="6">
+        <v>3</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="E57" s="6">
+        <f>IFERROR(INDEX('B6_Exercise_Library'!$D$4:$D$44,MATCH($D57,'B6_Exercise_Library'!$A$4:$A$44,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G57" s="6">
+        <v>5</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I57" s="6">
+        <v>35</v>
+      </c>
+      <c r="J57" s="6">
+        <v>8</v>
+      </c>
+      <c r="O57" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="P57" s="6">
+        <f>IF($B57="","",$B57&amp;"_W"&amp;$C57)</f>
         <v>0</v>
       </c>
     </row>
@@ -8366,7 +9180,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>575</v>
+        <v>594</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8377,20 +9191,20 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>576</v>
+        <v>595</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
-        <v>577</v>
+        <v>596</v>
       </c>
       <c r="B4" s="11">
         <v>80.8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>585</v>
+        <v>604</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
@@ -8399,21 +9213,21 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
-        <v>578</v>
+        <v>597</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>579</v>
+        <v>598</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="9" t="s">
-        <v>580</v>
+        <v>599</v>
       </c>
       <c r="B6" s="11">
         <v>2.2</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>586</v>
+        <v>605</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -8422,7 +9236,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
-        <v>581</v>
+        <v>600</v>
       </c>
       <c r="B7" s="11">
         <v>0.9</v>
@@ -8430,7 +9244,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
-        <v>582</v>
+        <v>601</v>
       </c>
       <c r="B8" s="10">
         <v>2700</v>
@@ -8438,7 +9252,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
-        <v>583</v>
+        <v>602</v>
       </c>
       <c r="B9" s="10">
         <f>ROUND(BW*B6,0)</f>
@@ -8447,7 +9261,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>584</v>
+        <v>603</v>
       </c>
       <c r="B10" s="10">
         <f>ROUND(BW*B7,0)</f>
@@ -8456,7 +9270,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>587</v>
+        <v>606</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -8470,27 +9284,27 @@
         <v>84</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>588</v>
+        <v>607</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>589</v>
+        <v>608</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>590</v>
+        <v>609</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>591</v>
+        <v>610</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>592</v>
+        <v>611</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>594</v>
+        <v>613</v>
       </c>
       <c r="B14" s="22">
         <v>250</v>
@@ -8512,7 +9326,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>595</v>
+        <v>614</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -8539,12 +9353,12 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>596</v>
+        <v>615</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>597</v>
+        <v>616</v>
       </c>
       <c r="B16" s="22">
         <v>200</v>
@@ -8566,12 +9380,12 @@
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>598</v>
+        <v>617</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
-        <v>599</v>
+        <v>618</v>
       </c>
       <c r="B17" s="22">
         <v>150</v>
@@ -8593,12 +9407,12 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>600</v>
+        <v>619</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
-        <v>601</v>
+        <v>620</v>
       </c>
       <c r="B18" s="22">
         <v>100</v>
@@ -8620,7 +9434,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>602</v>
+        <v>621</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8647,12 +9461,12 @@
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>603</v>
+        <v>622</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>604</v>
+        <v>623</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -8663,7 +9477,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>605</v>
+        <v>624</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -8674,7 +9488,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4" t="s">
-        <v>606</v>
+        <v>625</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -8685,7 +9499,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>607</v>
+        <v>626</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -8696,7 +9510,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -8741,7 +9555,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>609</v>
+        <v>628</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8750,7 +9564,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>610</v>
+        <v>629</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -8759,109 +9573,109 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="7" t="s">
-        <v>611</v>
+        <v>630</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>612</v>
+        <v>631</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>613</v>
+        <v>632</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>614</v>
+        <v>633</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>615</v>
+        <v>634</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="9" t="s">
-        <v>616</v>
+        <v>635</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>617</v>
+        <v>636</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>618</v>
+        <v>637</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>619</v>
+        <v>638</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>620</v>
+        <v>639</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>621</v>
+        <v>640</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>622</v>
+        <v>641</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>623</v>
+        <v>642</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>624</v>
+        <v>643</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>625</v>
+        <v>644</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="9" t="s">
-        <v>626</v>
+        <v>645</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>627</v>
+        <v>646</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>628</v>
+        <v>647</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>629</v>
+        <v>648</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>630</v>
+        <v>649</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>631</v>
+        <v>650</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>632</v>
+        <v>651</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>633</v>
+        <v>652</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>634</v>
+        <v>653</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>635</v>
+        <v>654</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="9" t="s">
-        <v>636</v>
+        <v>655</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>637</v>
+        <v>656</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>638</v>
+        <v>657</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>639</v>
+        <v>658</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>640</v>
+        <v>659</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
-        <v>641</v>
+        <v>660</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -8870,7 +9684,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="4" t="s">
-        <v>642</v>
+        <v>661</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -8879,7 +9693,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="4" t="s">
-        <v>643</v>
+        <v>662</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -8888,7 +9702,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="4" t="s">
-        <v>644</v>
+        <v>663</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -8897,7 +9711,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="4" t="s">
-        <v>645</v>
+        <v>664</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -8906,7 +9720,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="4" t="s">
-        <v>646</v>
+        <v>665</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -8915,7 +9729,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="4" t="s">
-        <v>647</v>
+        <v>666</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -8924,7 +9738,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
-        <v>648</v>
+        <v>667</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -8933,19 +9747,19 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="7" t="s">
-        <v>649</v>
+        <v>668</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>650</v>
+        <v>669</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>651</v>
+        <v>670</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>652</v>
+        <v>671</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>653</v>
+        <v>672</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -8953,16 +9767,16 @@
         <v>65</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>654</v>
+        <v>673</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>655</v>
+        <v>674</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>656</v>
+        <v>675</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>657</v>
+        <v>676</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -8970,16 +9784,16 @@
         <v>47</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>658</v>
+        <v>677</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>659</v>
+        <v>678</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>660</v>
+        <v>679</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>661</v>
+        <v>680</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -8987,16 +9801,16 @@
         <v>33</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>662</v>
+        <v>681</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>663</v>
+        <v>682</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>664</v>
+        <v>683</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>665</v>
+        <v>684</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -9004,21 +9818,21 @@
         <v>32</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>666</v>
+        <v>685</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>667</v>
+        <v>686</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>668</v>
+        <v>687</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>669</v>
+        <v>688</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="27" t="s">
-        <v>670</v>
+        <v>689</v>
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
@@ -9027,7 +9841,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="5" t="s">
-        <v>671</v>
+        <v>690</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -9036,7 +9850,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="4" t="s">
-        <v>672</v>
+        <v>691</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9045,7 +9859,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="4" t="s">
-        <v>673</v>
+        <v>692</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -9054,7 +9868,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="4" t="s">
-        <v>674</v>
+        <v>693</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -9063,7 +9877,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="4" t="s">
-        <v>675</v>
+        <v>694</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -9072,7 +9886,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="4" t="s">
-        <v>676</v>
+        <v>695</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -9081,7 +9895,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="5" t="s">
-        <v>677</v>
+        <v>696</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -9090,104 +9904,104 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="7" t="s">
-        <v>678</v>
+        <v>697</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>679</v>
+        <v>698</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>680</v>
+        <v>699</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="4" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="B36" s="28" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>683</v>
+        <v>702</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="4" t="s">
-        <v>684</v>
+        <v>703</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>685</v>
+        <v>704</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>686</v>
+        <v>705</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="4" t="s">
-        <v>687</v>
+        <v>706</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>688</v>
+        <v>707</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>689</v>
+        <v>708</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="4" t="s">
-        <v>690</v>
+        <v>709</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>691</v>
+        <v>710</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>692</v>
+        <v>711</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="4" t="s">
-        <v>690</v>
+        <v>709</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>693</v>
+        <v>712</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>694</v>
+        <v>713</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="4" t="s">
-        <v>695</v>
+        <v>714</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>696</v>
+        <v>715</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>697</v>
+        <v>716</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="4" t="s">
-        <v>698</v>
+        <v>717</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>699</v>
+        <v>718</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>700</v>
+        <v>719</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
@@ -9245,7 +10059,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>701</v>
+        <v>720</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9255,7 +10069,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="12" t="s">
-        <v>702</v>
+        <v>721</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -9280,12 +10094,12 @@
         <v>152</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>703</v>
+        <v>722</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>704</v>
+        <v>723</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Skill90",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)+SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Push",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9310,7 +10124,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>705</v>
+        <v>724</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Pull",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9335,7 +10149,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>706</v>
+        <v>725</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Legs",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9360,7 +10174,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>707</v>
+        <v>726</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIFS('B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9385,7 +10199,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>708</v>
+        <v>727</v>
       </c>
       <c r="B8" s="10">
         <f>SUMIFS('B6_Training_Log'!$N$2:$N$1000,'B6_Training_Log'!$D$2:$D$1000,"90",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9410,7 +10224,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>709</v>
+        <v>728</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"SkillOAHS",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9435,7 +10249,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>710</v>
+        <v>729</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTIFS('B6_Training_Log'!$E$2:$E$1000,"Planche",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9560,7 +10374,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="9" t="s">
-        <v>711</v>
+        <v>730</v>
       </c>
       <c r="B15" s="11">
         <f>SUMIFS('B6_Training_Log'!$G$2:$G$1000,'B6_Training_Log'!$E$2:$E$1000,"Core",'B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9585,7 +10399,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
-        <v>712</v>
+        <v>731</v>
       </c>
       <c r="B16" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$J$2:$J$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -9610,7 +10424,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9" t="s">
-        <v>713</v>
+        <v>732</v>
       </c>
       <c r="B17" s="11">
         <f>IFERROR(AVERAGEIFS('B6_Training_Log'!$K$2:$K$1000,'B6_Training_Log'!$C$2:$C$1000,1),0)</f>
@@ -9660,7 +10474,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>714</v>
+        <v>733</v>
       </c>
       <c r="B19" s="10">
         <f>COUNTIFS('B6_Training_Log'!$C$2:$C$1000,1)</f>
@@ -9704,7 +10518,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>715</v>
+        <v>734</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9712,7 +10526,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>716</v>
+        <v>735</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -9720,13 +10534,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
-        <v>717</v>
+        <v>736</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>718</v>
+        <v>737</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>719</v>
+        <v>738</v>
       </c>
       <c r="D4" s="7"/>
     </row>
@@ -9735,10 +10549,10 @@
         <v>523</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>720</v>
+        <v>739</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>721</v>
+        <v>740</v>
       </c>
       <c r="D5" s="4"/>
     </row>
@@ -9747,10 +10561,10 @@
         <v>524</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>722</v>
+        <v>741</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>723</v>
+        <v>742</v>
       </c>
       <c r="D6" s="4"/>
     </row>
@@ -9759,10 +10573,10 @@
         <v>525</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>724</v>
+        <v>743</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>725</v>
+        <v>744</v>
       </c>
       <c r="D7" s="4"/>
     </row>
@@ -9771,10 +10585,10 @@
         <v>359</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>726</v>
+        <v>745</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>727</v>
+        <v>746</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -9783,10 +10597,10 @@
         <v>362</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>728</v>
+        <v>747</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>729</v>
+        <v>748</v>
       </c>
       <c r="D9" s="4"/>
     </row>
@@ -9795,10 +10609,10 @@
         <v>526</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>730</v>
+        <v>749</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>731</v>
+        <v>750</v>
       </c>
       <c r="D10" s="4"/>
     </row>
@@ -9807,10 +10621,10 @@
         <v>527</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>733</v>
+        <v>752</v>
       </c>
       <c r="D11" s="4"/>
     </row>
@@ -9819,10 +10633,10 @@
         <v>528</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>735</v>
+        <v>754</v>
       </c>
       <c r="D12" s="4"/>
     </row>
@@ -9831,10 +10645,10 @@
         <v>529</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>736</v>
+        <v>755</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -9843,10 +10657,10 @@
         <v>530</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>737</v>
+        <v>756</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>738</v>
+        <v>757</v>
       </c>
       <c r="D14" s="4"/>
     </row>
@@ -9855,10 +10669,10 @@
         <v>531</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>739</v>
+        <v>758</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>740</v>
+        <v>759</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -9867,10 +10681,10 @@
         <v>532</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>741</v>
+        <v>760</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>742</v>
+        <v>761</v>
       </c>
       <c r="D16" s="4"/>
     </row>
@@ -9879,10 +10693,10 @@
         <v>533</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>743</v>
+        <v>762</v>
       </c>
       <c r="D17" s="4"/>
     </row>
@@ -9891,10 +10705,10 @@
         <v>534</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>744</v>
+        <v>763</v>
       </c>
       <c r="D18" s="4"/>
     </row>
@@ -9903,10 +10717,10 @@
         <v>91</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>745</v>
+        <v>764</v>
       </c>
       <c r="D19" s="4"/>
     </row>
@@ -9915,16 +10729,16 @@
         <v>535</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>746</v>
+        <v>765</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>747</v>
+        <v>766</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>748</v>
+        <v>767</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -9932,7 +10746,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>749</v>
+        <v>768</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -9940,7 +10754,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>750</v>
+        <v>769</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -9948,7 +10762,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>751</v>
+        <v>770</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -9956,7 +10770,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>752</v>
+        <v>771</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -9964,7 +10778,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>753</v>
+        <v>772</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -9972,7 +10786,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>754</v>
+        <v>773</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -9980,7 +10794,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
-        <v>755</v>
+        <v>774</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -9988,13 +10802,13 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>756</v>
+        <v>775</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>757</v>
+        <v>776</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>758</v>
+        <v>777</v>
       </c>
       <c r="D31" s="7"/>
     </row>
@@ -10003,10 +10817,10 @@
         <v>47</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>759</v>
+        <v>778</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>760</v>
+        <v>779</v>
       </c>
       <c r="D32" s="4"/>
     </row>
@@ -10015,10 +10829,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>761</v>
+        <v>780</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>762</v>
+        <v>781</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -10027,10 +10841,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>763</v>
+        <v>782</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>764</v>
+        <v>783</v>
       </c>
       <c r="D34" s="4"/>
     </row>
@@ -10039,22 +10853,22 @@
         <v>298</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>765</v>
+        <v>784</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>766</v>
+        <v>785</v>
       </c>
       <c r="D35" s="4"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="14" t="s">
-        <v>767</v>
+        <v>786</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>768</v>
+        <v>787</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>769</v>
+        <v>788</v>
       </c>
       <c r="D36" s="4"/>
     </row>
@@ -10063,16 +10877,16 @@
         <v>565</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>770</v>
+        <v>789</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>771</v>
+        <v>790</v>
       </c>
       <c r="D37" s="4"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
-        <v>772</v>
+        <v>791</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -10080,7 +10894,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>773</v>
+        <v>792</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -10088,7 +10902,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>774</v>
+        <v>793</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -10096,7 +10910,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>775</v>
+        <v>794</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -10104,7 +10918,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>776</v>
+        <v>795</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -10112,7 +10926,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>777</v>
+        <v>796</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -10120,7 +10934,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>778</v>
+        <v>797</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -10128,7 +10942,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>779</v>
+        <v>798</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>

</xml_diff>